<commit_message>
Updated via Streamlit Approval System
</commit_message>
<xml_diff>
--- a/PENDING_APPROVAL_SHEET.xlsx
+++ b/PENDING_APPROVAL_SHEET.xlsx
@@ -742,8 +742,16 @@
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
       <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK2" t="inlineStr"/>
       <c r="AL2" t="inlineStr"/>
       <c r="AM2" t="inlineStr"/>
@@ -857,8 +865,16 @@
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
       <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK3" t="inlineStr"/>
       <c r="AL3" t="inlineStr"/>
       <c r="AM3" t="inlineStr"/>
@@ -980,8 +996,16 @@
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr"/>
       <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="inlineStr"/>
       <c r="AM4" t="inlineStr"/>
@@ -1091,8 +1115,16 @@
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
       <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK5" t="inlineStr"/>
       <c r="AL5" t="inlineStr"/>
       <c r="AM5" t="inlineStr"/>
@@ -1202,8 +1234,16 @@
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
       <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK6" t="inlineStr"/>
       <c r="AL6" t="inlineStr"/>
       <c r="AM6" t="inlineStr"/>
@@ -1327,8 +1367,16 @@
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
       <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK7" t="inlineStr"/>
       <c r="AL7" t="inlineStr"/>
       <c r="AM7" t="inlineStr"/>
@@ -1452,8 +1500,16 @@
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
       <c r="AH8" t="inlineStr"/>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK8" t="inlineStr"/>
       <c r="AL8" t="inlineStr"/>
       <c r="AM8" t="inlineStr"/>
@@ -1577,8 +1633,16 @@
       <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="inlineStr"/>
-      <c r="AI9" t="inlineStr"/>
-      <c r="AJ9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK9" t="inlineStr"/>
       <c r="AL9" t="inlineStr"/>
       <c r="AM9" t="inlineStr"/>
@@ -1702,8 +1766,16 @@
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr"/>
       <c r="AH10" t="inlineStr"/>
-      <c r="AI10" t="inlineStr"/>
-      <c r="AJ10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK10" t="inlineStr"/>
       <c r="AL10" t="inlineStr"/>
       <c r="AM10" t="inlineStr"/>
@@ -1827,8 +1899,16 @@
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="inlineStr"/>
-      <c r="AI11" t="inlineStr"/>
-      <c r="AJ11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK11" t="inlineStr"/>
       <c r="AL11" t="inlineStr"/>
       <c r="AM11" t="inlineStr"/>
@@ -1940,8 +2020,16 @@
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr"/>
       <c r="AH12" t="inlineStr"/>
-      <c r="AI12" t="inlineStr"/>
-      <c r="AJ12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK12" t="inlineStr"/>
       <c r="AL12" t="inlineStr"/>
       <c r="AM12" t="inlineStr"/>
@@ -2051,8 +2139,16 @@
       <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr"/>
       <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr"/>
-      <c r="AJ13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK13" t="inlineStr"/>
       <c r="AL13" t="inlineStr"/>
       <c r="AM13" t="inlineStr"/>
@@ -2162,8 +2258,16 @@
       <c r="AF14" t="inlineStr"/>
       <c r="AG14" t="inlineStr"/>
       <c r="AH14" t="inlineStr"/>
-      <c r="AI14" t="inlineStr"/>
-      <c r="AJ14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK14" t="inlineStr"/>
       <c r="AL14" t="inlineStr"/>
       <c r="AM14" t="inlineStr"/>
@@ -2273,8 +2377,16 @@
       <c r="AF15" t="inlineStr"/>
       <c r="AG15" t="inlineStr"/>
       <c r="AH15" t="inlineStr"/>
-      <c r="AI15" t="inlineStr"/>
-      <c r="AJ15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK15" t="inlineStr"/>
       <c r="AL15" t="inlineStr"/>
       <c r="AM15" t="inlineStr"/>
@@ -2386,8 +2498,16 @@
       <c r="AF16" t="inlineStr"/>
       <c r="AG16" t="inlineStr"/>
       <c r="AH16" t="inlineStr"/>
-      <c r="AI16" t="inlineStr"/>
-      <c r="AJ16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK16" t="inlineStr"/>
       <c r="AL16" t="inlineStr"/>
       <c r="AM16" t="inlineStr"/>
@@ -2497,8 +2617,16 @@
       <c r="AF17" t="inlineStr"/>
       <c r="AG17" t="inlineStr"/>
       <c r="AH17" t="inlineStr"/>
-      <c r="AI17" t="inlineStr"/>
-      <c r="AJ17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK17" t="inlineStr"/>
       <c r="AL17" t="inlineStr"/>
       <c r="AM17" t="inlineStr"/>
@@ -2608,8 +2736,16 @@
       <c r="AF18" t="inlineStr"/>
       <c r="AG18" t="inlineStr"/>
       <c r="AH18" t="inlineStr"/>
-      <c r="AI18" t="inlineStr"/>
-      <c r="AJ18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK18" t="inlineStr"/>
       <c r="AL18" t="inlineStr"/>
       <c r="AM18" t="inlineStr"/>
@@ -2719,8 +2855,16 @@
       <c r="AF19" t="inlineStr"/>
       <c r="AG19" t="inlineStr"/>
       <c r="AH19" t="inlineStr"/>
-      <c r="AI19" t="inlineStr"/>
-      <c r="AJ19" t="inlineStr"/>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK19" t="inlineStr"/>
       <c r="AL19" t="inlineStr"/>
       <c r="AM19" t="inlineStr"/>
@@ -2844,8 +2988,16 @@
       <c r="AF20" t="inlineStr"/>
       <c r="AG20" t="inlineStr"/>
       <c r="AH20" t="inlineStr"/>
-      <c r="AI20" t="inlineStr"/>
-      <c r="AJ20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK20" t="inlineStr"/>
       <c r="AL20" t="inlineStr"/>
       <c r="AM20" t="inlineStr"/>
@@ -2955,8 +3107,16 @@
       <c r="AF21" t="inlineStr"/>
       <c r="AG21" t="inlineStr"/>
       <c r="AH21" t="inlineStr"/>
-      <c r="AI21" t="inlineStr"/>
-      <c r="AJ21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK21" t="inlineStr"/>
       <c r="AL21" t="inlineStr"/>
       <c r="AM21" t="inlineStr"/>
@@ -3066,8 +3226,16 @@
       <c r="AF22" t="inlineStr"/>
       <c r="AG22" t="inlineStr"/>
       <c r="AH22" t="inlineStr"/>
-      <c r="AI22" t="inlineStr"/>
-      <c r="AJ22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK22" t="inlineStr"/>
       <c r="AL22" t="inlineStr"/>
       <c r="AM22" t="inlineStr"/>
@@ -3177,8 +3345,16 @@
       <c r="AF23" t="inlineStr"/>
       <c r="AG23" t="inlineStr"/>
       <c r="AH23" t="inlineStr"/>
-      <c r="AI23" t="inlineStr"/>
-      <c r="AJ23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK23" t="inlineStr"/>
       <c r="AL23" t="inlineStr"/>
       <c r="AM23" t="inlineStr"/>
@@ -3290,8 +3466,16 @@
       <c r="AF24" t="inlineStr"/>
       <c r="AG24" t="inlineStr"/>
       <c r="AH24" t="inlineStr"/>
-      <c r="AI24" t="inlineStr"/>
-      <c r="AJ24" t="inlineStr"/>
+      <c r="AI24" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK24" t="inlineStr"/>
       <c r="AL24" t="inlineStr"/>
       <c r="AM24" t="inlineStr"/>
@@ -3401,8 +3585,16 @@
       <c r="AF25" t="inlineStr"/>
       <c r="AG25" t="inlineStr"/>
       <c r="AH25" t="inlineStr"/>
-      <c r="AI25" t="inlineStr"/>
-      <c r="AJ25" t="inlineStr"/>
+      <c r="AI25" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK25" t="inlineStr"/>
       <c r="AL25" t="inlineStr"/>
       <c r="AM25" t="inlineStr"/>
@@ -3512,8 +3704,16 @@
       <c r="AF26" t="inlineStr"/>
       <c r="AG26" t="inlineStr"/>
       <c r="AH26" t="inlineStr"/>
-      <c r="AI26" t="inlineStr"/>
-      <c r="AJ26" t="inlineStr"/>
+      <c r="AI26" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK26" t="inlineStr"/>
       <c r="AL26" t="inlineStr"/>
       <c r="AM26" t="inlineStr"/>
@@ -3637,8 +3837,16 @@
       <c r="AF27" t="inlineStr"/>
       <c r="AG27" t="inlineStr"/>
       <c r="AH27" t="inlineStr"/>
-      <c r="AI27" t="inlineStr"/>
-      <c r="AJ27" t="inlineStr"/>
+      <c r="AI27" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK27" t="inlineStr">
         <is>
           <t>HO</t>
@@ -3766,8 +3974,16 @@
       <c r="AF28" t="inlineStr"/>
       <c r="AG28" t="inlineStr"/>
       <c r="AH28" t="inlineStr"/>
-      <c r="AI28" t="inlineStr"/>
-      <c r="AJ28" t="inlineStr"/>
+      <c r="AI28" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK28" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -3895,8 +4111,16 @@
       <c r="AF29" t="inlineStr"/>
       <c r="AG29" t="inlineStr"/>
       <c r="AH29" t="inlineStr"/>
-      <c r="AI29" t="inlineStr"/>
-      <c r="AJ29" t="inlineStr"/>
+      <c r="AI29" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK29" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -4024,8 +4248,16 @@
       <c r="AF30" t="inlineStr"/>
       <c r="AG30" t="inlineStr"/>
       <c r="AH30" t="inlineStr"/>
-      <c r="AI30" t="inlineStr"/>
-      <c r="AJ30" t="inlineStr"/>
+      <c r="AI30" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ30" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK30" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -4113,8 +4345,16 @@
       <c r="AF31" t="inlineStr"/>
       <c r="AG31" t="inlineStr"/>
       <c r="AH31" t="inlineStr"/>
-      <c r="AI31" t="inlineStr"/>
-      <c r="AJ31" t="inlineStr"/>
+      <c r="AI31" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK31" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -4242,8 +4482,16 @@
       <c r="AF32" t="inlineStr"/>
       <c r="AG32" t="inlineStr"/>
       <c r="AH32" t="inlineStr"/>
-      <c r="AI32" t="inlineStr"/>
-      <c r="AJ32" t="inlineStr"/>
+      <c r="AI32" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK32" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -4371,8 +4619,16 @@
       <c r="AF33" t="inlineStr"/>
       <c r="AG33" t="inlineStr"/>
       <c r="AH33" t="inlineStr"/>
-      <c r="AI33" t="inlineStr"/>
-      <c r="AJ33" t="inlineStr"/>
+      <c r="AI33" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK33" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -4500,8 +4756,16 @@
       <c r="AF34" t="inlineStr"/>
       <c r="AG34" t="inlineStr"/>
       <c r="AH34" t="inlineStr"/>
-      <c r="AI34" t="inlineStr"/>
-      <c r="AJ34" t="inlineStr"/>
+      <c r="AI34" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ34" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK34" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -4629,8 +4893,16 @@
       <c r="AF35" t="inlineStr"/>
       <c r="AG35" t="inlineStr"/>
       <c r="AH35" t="inlineStr"/>
-      <c r="AI35" t="inlineStr"/>
-      <c r="AJ35" t="inlineStr"/>
+      <c r="AI35" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ35" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK35" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -4758,8 +5030,16 @@
       <c r="AF36" t="inlineStr"/>
       <c r="AG36" t="inlineStr"/>
       <c r="AH36" t="inlineStr"/>
-      <c r="AI36" t="inlineStr"/>
-      <c r="AJ36" t="inlineStr"/>
+      <c r="AI36" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ36" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK36" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -4887,8 +5167,16 @@
       <c r="AF37" t="inlineStr"/>
       <c r="AG37" t="inlineStr"/>
       <c r="AH37" t="inlineStr"/>
-      <c r="AI37" t="inlineStr"/>
-      <c r="AJ37" t="inlineStr"/>
+      <c r="AI37" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ37" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK37" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -5016,8 +5304,16 @@
       <c r="AF38" t="inlineStr"/>
       <c r="AG38" t="inlineStr"/>
       <c r="AH38" t="inlineStr"/>
-      <c r="AI38" t="inlineStr"/>
-      <c r="AJ38" t="inlineStr"/>
+      <c r="AI38" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ38" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK38" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -5135,8 +5431,16 @@
       <c r="AF39" t="inlineStr"/>
       <c r="AG39" t="inlineStr"/>
       <c r="AH39" t="inlineStr"/>
-      <c r="AI39" t="inlineStr"/>
-      <c r="AJ39" t="inlineStr"/>
+      <c r="AI39" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ39" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK39" t="inlineStr">
         <is>
           <t>HO</t>
@@ -5264,8 +5568,16 @@
       <c r="AF40" t="inlineStr"/>
       <c r="AG40" t="inlineStr"/>
       <c r="AH40" t="inlineStr"/>
-      <c r="AI40" t="inlineStr"/>
-      <c r="AJ40" t="inlineStr"/>
+      <c r="AI40" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ40" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK40" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -5389,8 +5701,16 @@
       <c r="AF41" t="inlineStr"/>
       <c r="AG41" t="inlineStr"/>
       <c r="AH41" t="inlineStr"/>
-      <c r="AI41" t="inlineStr"/>
-      <c r="AJ41" t="inlineStr"/>
+      <c r="AI41" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ41" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK41" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -5504,8 +5824,16 @@
       <c r="AF42" t="inlineStr"/>
       <c r="AG42" t="inlineStr"/>
       <c r="AH42" t="inlineStr"/>
-      <c r="AI42" t="inlineStr"/>
-      <c r="AJ42" t="inlineStr"/>
+      <c r="AI42" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ42" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK42" t="inlineStr"/>
       <c r="AL42" t="inlineStr"/>
       <c r="AM42" t="inlineStr"/>
@@ -5631,8 +5959,16 @@
       <c r="AF43" t="inlineStr"/>
       <c r="AG43" t="inlineStr"/>
       <c r="AH43" t="inlineStr"/>
-      <c r="AI43" t="inlineStr"/>
-      <c r="AJ43" t="inlineStr"/>
+      <c r="AI43" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ43" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK43" t="inlineStr"/>
       <c r="AL43" t="inlineStr"/>
       <c r="AM43" t="inlineStr"/>
@@ -5722,8 +6058,16 @@
       <c r="AF44" t="inlineStr"/>
       <c r="AG44" t="inlineStr"/>
       <c r="AH44" t="inlineStr"/>
-      <c r="AI44" t="inlineStr"/>
-      <c r="AJ44" t="inlineStr"/>
+      <c r="AI44" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ44" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK44" t="inlineStr"/>
       <c r="AL44" t="inlineStr"/>
       <c r="AM44" t="inlineStr"/>
@@ -5837,8 +6181,16 @@
       <c r="AF45" t="inlineStr"/>
       <c r="AG45" t="inlineStr"/>
       <c r="AH45" t="inlineStr"/>
-      <c r="AI45" t="inlineStr"/>
-      <c r="AJ45" t="inlineStr"/>
+      <c r="AI45" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ45" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK45" t="inlineStr"/>
       <c r="AL45" t="inlineStr"/>
       <c r="AM45" t="inlineStr"/>
@@ -5952,8 +6304,16 @@
       <c r="AF46" t="inlineStr"/>
       <c r="AG46" t="inlineStr"/>
       <c r="AH46" t="inlineStr"/>
-      <c r="AI46" t="inlineStr"/>
-      <c r="AJ46" t="inlineStr"/>
+      <c r="AI46" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ46" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK46" t="inlineStr"/>
       <c r="AL46" t="inlineStr"/>
       <c r="AM46" t="inlineStr"/>
@@ -6067,8 +6427,16 @@
       <c r="AF47" t="inlineStr"/>
       <c r="AG47" t="inlineStr"/>
       <c r="AH47" t="inlineStr"/>
-      <c r="AI47" t="inlineStr"/>
-      <c r="AJ47" t="inlineStr"/>
+      <c r="AI47" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ47" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK47" t="inlineStr"/>
       <c r="AL47" t="inlineStr"/>
       <c r="AM47" t="inlineStr"/>
@@ -6182,8 +6550,16 @@
       <c r="AF48" t="inlineStr"/>
       <c r="AG48" t="inlineStr"/>
       <c r="AH48" t="inlineStr"/>
-      <c r="AI48" t="inlineStr"/>
-      <c r="AJ48" t="inlineStr"/>
+      <c r="AI48" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ48" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK48" t="inlineStr"/>
       <c r="AL48" t="inlineStr"/>
       <c r="AM48" t="inlineStr"/>
@@ -6297,8 +6673,16 @@
       <c r="AF49" t="inlineStr"/>
       <c r="AG49" t="inlineStr"/>
       <c r="AH49" t="inlineStr"/>
-      <c r="AI49" t="inlineStr"/>
-      <c r="AJ49" t="inlineStr"/>
+      <c r="AI49" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ49" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK49" t="inlineStr"/>
       <c r="AL49" t="inlineStr"/>
       <c r="AM49" t="inlineStr"/>
@@ -6422,8 +6806,16 @@
       <c r="AF50" t="inlineStr"/>
       <c r="AG50" t="inlineStr"/>
       <c r="AH50" t="inlineStr"/>
-      <c r="AI50" t="inlineStr"/>
-      <c r="AJ50" t="inlineStr"/>
+      <c r="AI50" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ50" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK50" t="inlineStr">
         <is>
           <t>HO</t>
@@ -6551,8 +6943,16 @@
       <c r="AF51" t="inlineStr"/>
       <c r="AG51" t="inlineStr"/>
       <c r="AH51" t="inlineStr"/>
-      <c r="AI51" t="inlineStr"/>
-      <c r="AJ51" t="inlineStr"/>
+      <c r="AI51" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ51" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK51" t="inlineStr">
         <is>
           <t>HO</t>
@@ -6680,8 +7080,16 @@
       <c r="AF52" t="inlineStr"/>
       <c r="AG52" t="inlineStr"/>
       <c r="AH52" t="inlineStr"/>
-      <c r="AI52" t="inlineStr"/>
-      <c r="AJ52" t="inlineStr"/>
+      <c r="AI52" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ52" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK52" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -6809,8 +7217,16 @@
       <c r="AF53" t="inlineStr"/>
       <c r="AG53" t="inlineStr"/>
       <c r="AH53" t="inlineStr"/>
-      <c r="AI53" t="inlineStr"/>
-      <c r="AJ53" t="inlineStr"/>
+      <c r="AI53" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ53" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK53" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -6938,8 +7354,16 @@
       <c r="AF54" t="inlineStr"/>
       <c r="AG54" t="inlineStr"/>
       <c r="AH54" t="inlineStr"/>
-      <c r="AI54" t="inlineStr"/>
-      <c r="AJ54" t="inlineStr"/>
+      <c r="AI54" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ54" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK54" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -7053,8 +7477,16 @@
       <c r="AF55" t="inlineStr"/>
       <c r="AG55" t="inlineStr"/>
       <c r="AH55" t="inlineStr"/>
-      <c r="AI55" t="inlineStr"/>
-      <c r="AJ55" t="inlineStr"/>
+      <c r="AI55" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ55" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK55" t="inlineStr"/>
       <c r="AL55" t="inlineStr"/>
       <c r="AM55" t="inlineStr"/>
@@ -7164,8 +7596,16 @@
       <c r="AF56" t="inlineStr"/>
       <c r="AG56" t="inlineStr"/>
       <c r="AH56" t="inlineStr"/>
-      <c r="AI56" t="inlineStr"/>
-      <c r="AJ56" t="inlineStr"/>
+      <c r="AI56" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ56" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK56" t="inlineStr"/>
       <c r="AL56" t="inlineStr"/>
       <c r="AM56" t="inlineStr"/>
@@ -7275,8 +7715,16 @@
       <c r="AF57" t="inlineStr"/>
       <c r="AG57" t="inlineStr"/>
       <c r="AH57" t="inlineStr"/>
-      <c r="AI57" t="inlineStr"/>
-      <c r="AJ57" t="inlineStr"/>
+      <c r="AI57" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ57" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK57" t="inlineStr"/>
       <c r="AL57" t="inlineStr"/>
       <c r="AM57" t="inlineStr"/>
@@ -7386,8 +7834,16 @@
       <c r="AF58" t="inlineStr"/>
       <c r="AG58" t="inlineStr"/>
       <c r="AH58" t="inlineStr"/>
-      <c r="AI58" t="inlineStr"/>
-      <c r="AJ58" t="inlineStr"/>
+      <c r="AI58" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ58" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK58" t="inlineStr"/>
       <c r="AL58" t="inlineStr"/>
       <c r="AM58" t="inlineStr"/>
@@ -7497,8 +7953,16 @@
       <c r="AF59" t="inlineStr"/>
       <c r="AG59" t="inlineStr"/>
       <c r="AH59" t="inlineStr"/>
-      <c r="AI59" t="inlineStr"/>
-      <c r="AJ59" t="inlineStr"/>
+      <c r="AI59" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ59" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK59" t="inlineStr"/>
       <c r="AL59" t="inlineStr"/>
       <c r="AM59" t="inlineStr"/>
@@ -7608,8 +8072,16 @@
       <c r="AF60" t="inlineStr"/>
       <c r="AG60" t="inlineStr"/>
       <c r="AH60" t="inlineStr"/>
-      <c r="AI60" t="inlineStr"/>
-      <c r="AJ60" t="inlineStr"/>
+      <c r="AI60" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ60" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK60" t="inlineStr"/>
       <c r="AL60" t="inlineStr"/>
       <c r="AM60" t="inlineStr"/>
@@ -7733,8 +8205,16 @@
       <c r="AF61" t="inlineStr"/>
       <c r="AG61" t="inlineStr"/>
       <c r="AH61" t="inlineStr"/>
-      <c r="AI61" t="inlineStr"/>
-      <c r="AJ61" t="inlineStr"/>
+      <c r="AI61" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ61" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK61" t="inlineStr"/>
       <c r="AL61" t="inlineStr"/>
       <c r="AM61" t="inlineStr"/>
@@ -7846,8 +8326,16 @@
       <c r="AF62" t="inlineStr"/>
       <c r="AG62" t="inlineStr"/>
       <c r="AH62" t="inlineStr"/>
-      <c r="AI62" t="inlineStr"/>
-      <c r="AJ62" t="inlineStr"/>
+      <c r="AI62" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ62" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK62" t="inlineStr"/>
       <c r="AL62" t="inlineStr"/>
       <c r="AM62" t="inlineStr"/>
@@ -7957,8 +8445,16 @@
       <c r="AF63" t="inlineStr"/>
       <c r="AG63" t="inlineStr"/>
       <c r="AH63" t="inlineStr"/>
-      <c r="AI63" t="inlineStr"/>
-      <c r="AJ63" t="inlineStr"/>
+      <c r="AI63" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ63" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK63" t="inlineStr"/>
       <c r="AL63" t="inlineStr"/>
       <c r="AM63" t="inlineStr"/>
@@ -8068,8 +8564,16 @@
       <c r="AF64" t="inlineStr"/>
       <c r="AG64" t="inlineStr"/>
       <c r="AH64" t="inlineStr"/>
-      <c r="AI64" t="inlineStr"/>
-      <c r="AJ64" t="inlineStr"/>
+      <c r="AI64" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ64" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK64" t="inlineStr"/>
       <c r="AL64" t="inlineStr"/>
       <c r="AM64" t="inlineStr"/>
@@ -8179,8 +8683,16 @@
       <c r="AF65" t="inlineStr"/>
       <c r="AG65" t="inlineStr"/>
       <c r="AH65" t="inlineStr"/>
-      <c r="AI65" t="inlineStr"/>
-      <c r="AJ65" t="inlineStr"/>
+      <c r="AI65" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ65" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK65" t="inlineStr"/>
       <c r="AL65" t="inlineStr"/>
       <c r="AM65" t="inlineStr"/>
@@ -8292,8 +8804,16 @@
       <c r="AF66" t="inlineStr"/>
       <c r="AG66" t="inlineStr"/>
       <c r="AH66" t="inlineStr"/>
-      <c r="AI66" t="inlineStr"/>
-      <c r="AJ66" t="inlineStr"/>
+      <c r="AI66" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ66" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK66" t="inlineStr"/>
       <c r="AL66" t="inlineStr"/>
       <c r="AM66" t="inlineStr"/>
@@ -8403,8 +8923,16 @@
       <c r="AF67" t="inlineStr"/>
       <c r="AG67" t="inlineStr"/>
       <c r="AH67" t="inlineStr"/>
-      <c r="AI67" t="inlineStr"/>
-      <c r="AJ67" t="inlineStr"/>
+      <c r="AI67" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ67" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK67" t="inlineStr"/>
       <c r="AL67" t="inlineStr"/>
       <c r="AM67" t="inlineStr"/>
@@ -8516,8 +9044,16 @@
       <c r="AF68" t="inlineStr"/>
       <c r="AG68" t="inlineStr"/>
       <c r="AH68" t="inlineStr"/>
-      <c r="AI68" t="inlineStr"/>
-      <c r="AJ68" t="inlineStr"/>
+      <c r="AI68" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ68" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK68" t="inlineStr"/>
       <c r="AL68" t="inlineStr"/>
       <c r="AM68" t="inlineStr"/>
@@ -8627,8 +9163,16 @@
       <c r="AF69" t="inlineStr"/>
       <c r="AG69" t="inlineStr"/>
       <c r="AH69" t="inlineStr"/>
-      <c r="AI69" t="inlineStr"/>
-      <c r="AJ69" t="inlineStr"/>
+      <c r="AI69" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ69" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK69" t="inlineStr"/>
       <c r="AL69" t="inlineStr"/>
       <c r="AM69" t="inlineStr"/>
@@ -8740,8 +9284,16 @@
       <c r="AF70" t="inlineStr"/>
       <c r="AG70" t="inlineStr"/>
       <c r="AH70" t="inlineStr"/>
-      <c r="AI70" t="inlineStr"/>
-      <c r="AJ70" t="inlineStr"/>
+      <c r="AI70" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ70" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK70" t="inlineStr"/>
       <c r="AL70" t="inlineStr"/>
       <c r="AM70" t="inlineStr"/>
@@ -8851,8 +9403,16 @@
       <c r="AF71" t="inlineStr"/>
       <c r="AG71" t="inlineStr"/>
       <c r="AH71" t="inlineStr"/>
-      <c r="AI71" t="inlineStr"/>
-      <c r="AJ71" t="inlineStr"/>
+      <c r="AI71" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ71" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK71" t="inlineStr"/>
       <c r="AL71" t="inlineStr"/>
       <c r="AM71" t="inlineStr"/>
@@ -8972,8 +9532,16 @@
       <c r="AF72" t="inlineStr"/>
       <c r="AG72" t="inlineStr"/>
       <c r="AH72" t="inlineStr"/>
-      <c r="AI72" t="inlineStr"/>
-      <c r="AJ72" t="inlineStr"/>
+      <c r="AI72" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ72" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK72" t="inlineStr"/>
       <c r="AL72" t="inlineStr"/>
       <c r="AM72" t="inlineStr"/>
@@ -9087,8 +9655,16 @@
       <c r="AF73" t="inlineStr"/>
       <c r="AG73" t="inlineStr"/>
       <c r="AH73" t="inlineStr"/>
-      <c r="AI73" t="inlineStr"/>
-      <c r="AJ73" t="inlineStr"/>
+      <c r="AI73" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ73" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK73" t="inlineStr"/>
       <c r="AL73" t="inlineStr"/>
       <c r="AM73" t="inlineStr"/>
@@ -9202,8 +9778,16 @@
       <c r="AF74" t="inlineStr"/>
       <c r="AG74" t="inlineStr"/>
       <c r="AH74" t="inlineStr"/>
-      <c r="AI74" t="inlineStr"/>
-      <c r="AJ74" t="inlineStr"/>
+      <c r="AI74" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ74" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK74" t="inlineStr"/>
       <c r="AL74" t="inlineStr"/>
       <c r="AM74" t="inlineStr"/>
@@ -9317,8 +9901,16 @@
       <c r="AF75" t="inlineStr"/>
       <c r="AG75" t="inlineStr"/>
       <c r="AH75" t="inlineStr"/>
-      <c r="AI75" t="inlineStr"/>
-      <c r="AJ75" t="inlineStr"/>
+      <c r="AI75" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ75" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK75" t="inlineStr"/>
       <c r="AL75" t="inlineStr"/>
       <c r="AM75" t="inlineStr"/>
@@ -9432,8 +10024,16 @@
       <c r="AF76" t="inlineStr"/>
       <c r="AG76" t="inlineStr"/>
       <c r="AH76" t="inlineStr"/>
-      <c r="AI76" t="inlineStr"/>
-      <c r="AJ76" t="inlineStr"/>
+      <c r="AI76" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ76" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK76" t="inlineStr"/>
       <c r="AL76" t="inlineStr"/>
       <c r="AM76" t="inlineStr"/>
@@ -9543,8 +10143,16 @@
       <c r="AF77" t="inlineStr"/>
       <c r="AG77" t="inlineStr"/>
       <c r="AH77" t="inlineStr"/>
-      <c r="AI77" t="inlineStr"/>
-      <c r="AJ77" t="inlineStr"/>
+      <c r="AI77" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ77" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK77" t="inlineStr"/>
       <c r="AL77" t="inlineStr"/>
       <c r="AM77" t="inlineStr"/>
@@ -9656,8 +10264,16 @@
       <c r="AF78" t="inlineStr"/>
       <c r="AG78" t="inlineStr"/>
       <c r="AH78" t="inlineStr"/>
-      <c r="AI78" t="inlineStr"/>
-      <c r="AJ78" t="inlineStr"/>
+      <c r="AI78" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ78" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK78" t="inlineStr"/>
       <c r="AL78" t="inlineStr"/>
       <c r="AM78" t="inlineStr"/>
@@ -9769,8 +10385,16 @@
       <c r="AF79" t="inlineStr"/>
       <c r="AG79" t="inlineStr"/>
       <c r="AH79" t="inlineStr"/>
-      <c r="AI79" t="inlineStr"/>
-      <c r="AJ79" t="inlineStr"/>
+      <c r="AI79" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ79" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK79" t="inlineStr"/>
       <c r="AL79" t="inlineStr"/>
       <c r="AM79" t="inlineStr"/>
@@ -9882,8 +10506,16 @@
       <c r="AF80" t="inlineStr"/>
       <c r="AG80" t="inlineStr"/>
       <c r="AH80" t="inlineStr"/>
-      <c r="AI80" t="inlineStr"/>
-      <c r="AJ80" t="inlineStr"/>
+      <c r="AI80" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ80" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK80" t="inlineStr"/>
       <c r="AL80" t="inlineStr"/>
       <c r="AM80" t="inlineStr"/>
@@ -9995,8 +10627,16 @@
       <c r="AF81" t="inlineStr"/>
       <c r="AG81" t="inlineStr"/>
       <c r="AH81" t="inlineStr"/>
-      <c r="AI81" t="inlineStr"/>
-      <c r="AJ81" t="inlineStr"/>
+      <c r="AI81" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ81" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK81" t="inlineStr"/>
       <c r="AL81" t="inlineStr"/>
       <c r="AM81" t="inlineStr"/>
@@ -10108,8 +10748,16 @@
       <c r="AF82" t="inlineStr"/>
       <c r="AG82" t="inlineStr"/>
       <c r="AH82" t="inlineStr"/>
-      <c r="AI82" t="inlineStr"/>
-      <c r="AJ82" t="inlineStr"/>
+      <c r="AI82" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ82" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK82" t="inlineStr"/>
       <c r="AL82" t="inlineStr"/>
       <c r="AM82" t="inlineStr"/>
@@ -10233,8 +10881,16 @@
       <c r="AF83" t="inlineStr"/>
       <c r="AG83" t="inlineStr"/>
       <c r="AH83" t="inlineStr"/>
-      <c r="AI83" t="inlineStr"/>
-      <c r="AJ83" t="inlineStr"/>
+      <c r="AI83" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ83" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK83" t="inlineStr"/>
       <c r="AL83" t="inlineStr"/>
       <c r="AM83" t="inlineStr"/>
@@ -10346,8 +11002,16 @@
       <c r="AF84" t="inlineStr"/>
       <c r="AG84" t="inlineStr"/>
       <c r="AH84" t="inlineStr"/>
-      <c r="AI84" t="inlineStr"/>
-      <c r="AJ84" t="inlineStr"/>
+      <c r="AI84" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ84" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK84" t="inlineStr"/>
       <c r="AL84" t="inlineStr"/>
       <c r="AM84" t="inlineStr"/>
@@ -10459,8 +11123,16 @@
       <c r="AF85" t="inlineStr"/>
       <c r="AG85" t="inlineStr"/>
       <c r="AH85" t="inlineStr"/>
-      <c r="AI85" t="inlineStr"/>
-      <c r="AJ85" t="inlineStr"/>
+      <c r="AI85" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ85" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK85" t="inlineStr"/>
       <c r="AL85" t="inlineStr"/>
       <c r="AM85" t="inlineStr"/>
@@ -10572,8 +11244,16 @@
       <c r="AF86" t="inlineStr"/>
       <c r="AG86" t="inlineStr"/>
       <c r="AH86" t="inlineStr"/>
-      <c r="AI86" t="inlineStr"/>
-      <c r="AJ86" t="inlineStr"/>
+      <c r="AI86" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ86" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK86" t="inlineStr"/>
       <c r="AL86" t="inlineStr"/>
       <c r="AM86" t="inlineStr"/>
@@ -10685,8 +11365,16 @@
       <c r="AF87" t="inlineStr"/>
       <c r="AG87" t="inlineStr"/>
       <c r="AH87" t="inlineStr"/>
-      <c r="AI87" t="inlineStr"/>
-      <c r="AJ87" t="inlineStr"/>
+      <c r="AI87" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ87" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK87" t="inlineStr"/>
       <c r="AL87" t="inlineStr"/>
       <c r="AM87" t="inlineStr"/>
@@ -10798,8 +11486,16 @@
       <c r="AF88" t="inlineStr"/>
       <c r="AG88" t="inlineStr"/>
       <c r="AH88" t="inlineStr"/>
-      <c r="AI88" t="inlineStr"/>
-      <c r="AJ88" t="inlineStr"/>
+      <c r="AI88" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ88" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK88" t="inlineStr"/>
       <c r="AL88" t="inlineStr"/>
       <c r="AM88" t="inlineStr"/>
@@ -10909,8 +11605,16 @@
       <c r="AF89" t="inlineStr"/>
       <c r="AG89" t="inlineStr"/>
       <c r="AH89" t="inlineStr"/>
-      <c r="AI89" t="inlineStr"/>
-      <c r="AJ89" t="inlineStr"/>
+      <c r="AI89" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ89" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK89" t="inlineStr"/>
       <c r="AL89" t="inlineStr"/>
       <c r="AM89" t="inlineStr"/>
@@ -11022,8 +11726,16 @@
       <c r="AF90" t="inlineStr"/>
       <c r="AG90" t="inlineStr"/>
       <c r="AH90" t="inlineStr"/>
-      <c r="AI90" t="inlineStr"/>
-      <c r="AJ90" t="inlineStr"/>
+      <c r="AI90" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ90" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK90" t="inlineStr"/>
       <c r="AL90" t="inlineStr"/>
       <c r="AM90" t="inlineStr"/>
@@ -11133,8 +11845,16 @@
       <c r="AF91" t="inlineStr"/>
       <c r="AG91" t="inlineStr"/>
       <c r="AH91" t="inlineStr"/>
-      <c r="AI91" t="inlineStr"/>
-      <c r="AJ91" t="inlineStr"/>
+      <c r="AI91" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ91" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK91" t="inlineStr"/>
       <c r="AL91" t="inlineStr"/>
       <c r="AM91" t="inlineStr"/>
@@ -11246,8 +11966,16 @@
       <c r="AF92" t="inlineStr"/>
       <c r="AG92" t="inlineStr"/>
       <c r="AH92" t="inlineStr"/>
-      <c r="AI92" t="inlineStr"/>
-      <c r="AJ92" t="inlineStr"/>
+      <c r="AI92" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ92" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK92" t="inlineStr"/>
       <c r="AL92" t="inlineStr"/>
       <c r="AM92" t="inlineStr"/>
@@ -11357,8 +12085,16 @@
       <c r="AF93" t="inlineStr"/>
       <c r="AG93" t="inlineStr"/>
       <c r="AH93" t="inlineStr"/>
-      <c r="AI93" t="inlineStr"/>
-      <c r="AJ93" t="inlineStr"/>
+      <c r="AI93" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ93" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK93" t="inlineStr"/>
       <c r="AL93" t="inlineStr"/>
       <c r="AM93" t="inlineStr"/>
@@ -11478,8 +12214,16 @@
       <c r="AF94" t="inlineStr"/>
       <c r="AG94" t="inlineStr"/>
       <c r="AH94" t="inlineStr"/>
-      <c r="AI94" t="inlineStr"/>
-      <c r="AJ94" t="inlineStr"/>
+      <c r="AI94" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ94" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK94" t="inlineStr"/>
       <c r="AL94" t="inlineStr"/>
       <c r="AM94" t="inlineStr"/>
@@ -11589,8 +12333,16 @@
       <c r="AF95" t="inlineStr"/>
       <c r="AG95" t="inlineStr"/>
       <c r="AH95" t="inlineStr"/>
-      <c r="AI95" t="inlineStr"/>
-      <c r="AJ95" t="inlineStr"/>
+      <c r="AI95" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ95" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK95" t="inlineStr"/>
       <c r="AL95" t="inlineStr"/>
       <c r="AM95" t="inlineStr"/>
@@ -11700,8 +12452,16 @@
       <c r="AF96" t="inlineStr"/>
       <c r="AG96" t="inlineStr"/>
       <c r="AH96" t="inlineStr"/>
-      <c r="AI96" t="inlineStr"/>
-      <c r="AJ96" t="inlineStr"/>
+      <c r="AI96" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ96" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK96" t="inlineStr"/>
       <c r="AL96" t="inlineStr"/>
       <c r="AM96" t="inlineStr"/>
@@ -11825,8 +12585,16 @@
       <c r="AF97" t="inlineStr"/>
       <c r="AG97" t="inlineStr"/>
       <c r="AH97" t="inlineStr"/>
-      <c r="AI97" t="inlineStr"/>
-      <c r="AJ97" t="inlineStr"/>
+      <c r="AI97" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ97" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK97" t="inlineStr"/>
       <c r="AL97" t="inlineStr"/>
       <c r="AM97" t="inlineStr"/>
@@ -11950,8 +12718,16 @@
       <c r="AF98" t="inlineStr"/>
       <c r="AG98" t="inlineStr"/>
       <c r="AH98" t="inlineStr"/>
-      <c r="AI98" t="inlineStr"/>
-      <c r="AJ98" t="inlineStr"/>
+      <c r="AI98" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ98" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK98" t="inlineStr"/>
       <c r="AL98" t="inlineStr"/>
       <c r="AM98" t="inlineStr"/>
@@ -12075,8 +12851,16 @@
       <c r="AF99" t="inlineStr"/>
       <c r="AG99" t="inlineStr"/>
       <c r="AH99" t="inlineStr"/>
-      <c r="AI99" t="inlineStr"/>
-      <c r="AJ99" t="inlineStr"/>
+      <c r="AI99" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ99" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK99" t="inlineStr"/>
       <c r="AL99" t="inlineStr"/>
       <c r="AM99" t="inlineStr"/>
@@ -12200,8 +12984,16 @@
       <c r="AF100" t="inlineStr"/>
       <c r="AG100" t="inlineStr"/>
       <c r="AH100" t="inlineStr"/>
-      <c r="AI100" t="inlineStr"/>
-      <c r="AJ100" t="inlineStr"/>
+      <c r="AI100" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ100" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK100" t="inlineStr"/>
       <c r="AL100" t="inlineStr"/>
       <c r="AM100" t="inlineStr"/>
@@ -12325,8 +13117,16 @@
       <c r="AF101" t="inlineStr"/>
       <c r="AG101" t="inlineStr"/>
       <c r="AH101" t="inlineStr"/>
-      <c r="AI101" t="inlineStr"/>
-      <c r="AJ101" t="inlineStr"/>
+      <c r="AI101" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ101" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK101" t="inlineStr">
         <is>
           <t>IOCL FEROKE</t>
@@ -12450,8 +13250,16 @@
       <c r="AF102" t="inlineStr"/>
       <c r="AG102" t="inlineStr"/>
       <c r="AH102" t="inlineStr"/>
-      <c r="AI102" t="inlineStr"/>
-      <c r="AJ102" t="inlineStr"/>
+      <c r="AI102" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ102" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK102" t="inlineStr">
         <is>
           <t>IOCL FEROKE</t>
@@ -12579,8 +13387,16 @@
       <c r="AF103" t="inlineStr"/>
       <c r="AG103" t="inlineStr"/>
       <c r="AH103" t="inlineStr"/>
-      <c r="AI103" t="inlineStr"/>
-      <c r="AJ103" t="inlineStr"/>
+      <c r="AI103" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ103" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK103" t="inlineStr">
         <is>
           <t>HO</t>
@@ -12708,8 +13524,16 @@
       <c r="AF104" t="inlineStr"/>
       <c r="AG104" t="inlineStr"/>
       <c r="AH104" t="inlineStr"/>
-      <c r="AI104" t="inlineStr"/>
-      <c r="AJ104" t="inlineStr"/>
+      <c r="AI104" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ104" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK104" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -12837,8 +13661,16 @@
       <c r="AF105" t="inlineStr"/>
       <c r="AG105" t="inlineStr"/>
       <c r="AH105" t="inlineStr"/>
-      <c r="AI105" t="inlineStr"/>
-      <c r="AJ105" t="inlineStr"/>
+      <c r="AI105" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ105" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK105" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -12966,8 +13798,16 @@
       <c r="AF106" t="inlineStr"/>
       <c r="AG106" t="inlineStr"/>
       <c r="AH106" t="inlineStr"/>
-      <c r="AI106" t="inlineStr"/>
-      <c r="AJ106" t="inlineStr"/>
+      <c r="AI106" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ106" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK106" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -13055,8 +13895,16 @@
       <c r="AF107" t="inlineStr"/>
       <c r="AG107" t="inlineStr"/>
       <c r="AH107" t="inlineStr"/>
-      <c r="AI107" t="inlineStr"/>
-      <c r="AJ107" t="inlineStr"/>
+      <c r="AI107" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ107" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK107" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -13184,8 +14032,16 @@
       <c r="AF108" t="inlineStr"/>
       <c r="AG108" t="inlineStr"/>
       <c r="AH108" t="inlineStr"/>
-      <c r="AI108" t="inlineStr"/>
-      <c r="AJ108" t="inlineStr"/>
+      <c r="AI108" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ108" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK108" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -13313,8 +14169,16 @@
       <c r="AF109" t="inlineStr"/>
       <c r="AG109" t="inlineStr"/>
       <c r="AH109" t="inlineStr"/>
-      <c r="AI109" t="inlineStr"/>
-      <c r="AJ109" t="inlineStr"/>
+      <c r="AI109" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ109" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK109" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -13442,8 +14306,16 @@
       <c r="AF110" t="inlineStr"/>
       <c r="AG110" t="inlineStr"/>
       <c r="AH110" t="inlineStr"/>
-      <c r="AI110" t="inlineStr"/>
-      <c r="AJ110" t="inlineStr"/>
+      <c r="AI110" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ110" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK110" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -13571,8 +14443,16 @@
       <c r="AF111" t="inlineStr"/>
       <c r="AG111" t="inlineStr"/>
       <c r="AH111" t="inlineStr"/>
-      <c r="AI111" t="inlineStr"/>
-      <c r="AJ111" t="inlineStr"/>
+      <c r="AI111" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ111" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK111" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -13700,8 +14580,16 @@
       <c r="AF112" t="inlineStr"/>
       <c r="AG112" t="inlineStr"/>
       <c r="AH112" t="inlineStr"/>
-      <c r="AI112" t="inlineStr"/>
-      <c r="AJ112" t="inlineStr"/>
+      <c r="AI112" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ112" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK112" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -13829,8 +14717,16 @@
       <c r="AF113" t="inlineStr"/>
       <c r="AG113" t="inlineStr"/>
       <c r="AH113" t="inlineStr"/>
-      <c r="AI113" t="inlineStr"/>
-      <c r="AJ113" t="inlineStr"/>
+      <c r="AI113" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ113" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK113" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -13958,8 +14854,16 @@
       <c r="AF114" t="inlineStr"/>
       <c r="AG114" t="inlineStr"/>
       <c r="AH114" t="inlineStr"/>
-      <c r="AI114" t="inlineStr"/>
-      <c r="AJ114" t="inlineStr"/>
+      <c r="AI114" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ114" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK114" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -14087,8 +14991,16 @@
       <c r="AF115" t="inlineStr"/>
       <c r="AG115" t="inlineStr"/>
       <c r="AH115" t="inlineStr"/>
-      <c r="AI115" t="inlineStr"/>
-      <c r="AJ115" t="inlineStr"/>
+      <c r="AI115" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ115" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK115" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -14212,8 +15124,16 @@
       <c r="AF116" t="inlineStr"/>
       <c r="AG116" t="inlineStr"/>
       <c r="AH116" t="inlineStr"/>
-      <c r="AI116" t="inlineStr"/>
-      <c r="AJ116" t="inlineStr"/>
+      <c r="AI116" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ116" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK116" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -14341,8 +15261,16 @@
       <c r="AF117" t="inlineStr"/>
       <c r="AG117" t="inlineStr"/>
       <c r="AH117" t="inlineStr"/>
-      <c r="AI117" t="inlineStr"/>
-      <c r="AJ117" t="inlineStr"/>
+      <c r="AI117" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ117" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK117" t="inlineStr">
         <is>
           <t>HO</t>
@@ -14470,8 +15398,16 @@
       <c r="AF118" t="inlineStr"/>
       <c r="AG118" t="inlineStr"/>
       <c r="AH118" t="inlineStr"/>
-      <c r="AI118" t="inlineStr"/>
-      <c r="AJ118" t="inlineStr"/>
+      <c r="AI118" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ118" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK118" t="inlineStr">
         <is>
           <t>HO</t>
@@ -14599,8 +15535,16 @@
       <c r="AF119" t="inlineStr"/>
       <c r="AG119" t="inlineStr"/>
       <c r="AH119" t="inlineStr"/>
-      <c r="AI119" t="inlineStr"/>
-      <c r="AJ119" t="inlineStr"/>
+      <c r="AI119" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ119" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK119" t="inlineStr">
         <is>
           <t>BELLARI</t>
@@ -14728,8 +15672,16 @@
       <c r="AF120" t="inlineStr"/>
       <c r="AG120" t="inlineStr"/>
       <c r="AH120" t="inlineStr"/>
-      <c r="AI120" t="inlineStr"/>
-      <c r="AJ120" t="inlineStr"/>
+      <c r="AI120" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ120" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK120" t="inlineStr">
         <is>
           <t>IOCL FEROKE</t>
@@ -14857,8 +15809,16 @@
       <c r="AF121" t="inlineStr"/>
       <c r="AG121" t="inlineStr"/>
       <c r="AH121" t="inlineStr"/>
-      <c r="AI121" t="inlineStr"/>
-      <c r="AJ121" t="inlineStr"/>
+      <c r="AI121" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ121" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK121" t="inlineStr">
         <is>
           <t>ONGC IPSHEM</t>
@@ -14986,8 +15946,16 @@
       <c r="AF122" t="inlineStr"/>
       <c r="AG122" t="inlineStr"/>
       <c r="AH122" t="inlineStr"/>
-      <c r="AI122" t="inlineStr"/>
-      <c r="AJ122" t="inlineStr"/>
+      <c r="AI122" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ122" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK122" t="inlineStr">
         <is>
           <t>ONGC IPSHEM</t>
@@ -15115,8 +16083,16 @@
       <c r="AF123" t="inlineStr"/>
       <c r="AG123" t="inlineStr"/>
       <c r="AH123" t="inlineStr"/>
-      <c r="AI123" t="inlineStr"/>
-      <c r="AJ123" t="inlineStr"/>
+      <c r="AI123" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ123" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK123" t="inlineStr">
         <is>
           <t>ONGC IPSHEM</t>
@@ -15244,8 +16220,16 @@
       <c r="AF124" t="inlineStr"/>
       <c r="AG124" t="inlineStr"/>
       <c r="AH124" t="inlineStr"/>
-      <c r="AI124" t="inlineStr"/>
-      <c r="AJ124" t="inlineStr"/>
+      <c r="AI124" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ124" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK124" t="inlineStr">
         <is>
           <t>ONGC IPSHEM</t>
@@ -15373,8 +16357,16 @@
       <c r="AF125" t="inlineStr"/>
       <c r="AG125" t="inlineStr"/>
       <c r="AH125" t="inlineStr"/>
-      <c r="AI125" t="inlineStr"/>
-      <c r="AJ125" t="inlineStr"/>
+      <c r="AI125" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ125" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK125" t="inlineStr">
         <is>
           <t>ONGC IPSHEM</t>
@@ -15502,8 +16494,16 @@
       <c r="AF126" t="inlineStr"/>
       <c r="AG126" t="inlineStr"/>
       <c r="AH126" t="inlineStr"/>
-      <c r="AI126" t="inlineStr"/>
-      <c r="AJ126" t="inlineStr"/>
+      <c r="AI126" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ126" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK126" t="inlineStr">
         <is>
           <t>ONGC IPSHEM</t>
@@ -15631,8 +16631,16 @@
       <c r="AF127" t="inlineStr"/>
       <c r="AG127" t="inlineStr"/>
       <c r="AH127" t="inlineStr"/>
-      <c r="AI127" t="inlineStr"/>
-      <c r="AJ127" t="inlineStr"/>
+      <c r="AI127" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ127" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK127" t="inlineStr">
         <is>
           <t>ONGC IPSHEM</t>
@@ -15760,8 +16768,16 @@
       <c r="AF128" t="inlineStr"/>
       <c r="AG128" t="inlineStr"/>
       <c r="AH128" t="inlineStr"/>
-      <c r="AI128" t="inlineStr"/>
-      <c r="AJ128" t="inlineStr"/>
+      <c r="AI128" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ128" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK128" t="inlineStr">
         <is>
           <t>ONGC IPSHEM</t>
@@ -15889,8 +16905,16 @@
       <c r="AF129" t="inlineStr"/>
       <c r="AG129" t="inlineStr"/>
       <c r="AH129" t="inlineStr"/>
-      <c r="AI129" t="inlineStr"/>
-      <c r="AJ129" t="inlineStr"/>
+      <c r="AI129" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ129" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK129" t="inlineStr">
         <is>
           <t>ONGC IPSHEM</t>
@@ -16018,8 +17042,16 @@
       <c r="AF130" t="inlineStr"/>
       <c r="AG130" t="inlineStr"/>
       <c r="AH130" t="inlineStr"/>
-      <c r="AI130" t="inlineStr"/>
-      <c r="AJ130" t="inlineStr"/>
+      <c r="AI130" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ130" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK130" t="inlineStr">
         <is>
           <t>BELLARI</t>
@@ -16147,8 +17179,16 @@
       <c r="AF131" t="inlineStr"/>
       <c r="AG131" t="inlineStr"/>
       <c r="AH131" t="inlineStr"/>
-      <c r="AI131" t="inlineStr"/>
-      <c r="AJ131" t="inlineStr"/>
+      <c r="AI131" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ131" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK131" t="inlineStr">
         <is>
           <t>BELLARI</t>
@@ -16276,8 +17316,16 @@
       <c r="AF132" t="inlineStr"/>
       <c r="AG132" t="inlineStr"/>
       <c r="AH132" t="inlineStr"/>
-      <c r="AI132" t="inlineStr"/>
-      <c r="AJ132" t="inlineStr"/>
+      <c r="AI132" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ132" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK132" t="inlineStr">
         <is>
           <t>BELLARI</t>
@@ -16405,8 +17453,16 @@
       <c r="AF133" t="inlineStr"/>
       <c r="AG133" t="inlineStr"/>
       <c r="AH133" t="inlineStr"/>
-      <c r="AI133" t="inlineStr"/>
-      <c r="AJ133" t="inlineStr"/>
+      <c r="AI133" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ133" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK133" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -16534,8 +17590,16 @@
       <c r="AF134" t="inlineStr"/>
       <c r="AG134" t="inlineStr"/>
       <c r="AH134" t="inlineStr"/>
-      <c r="AI134" t="inlineStr"/>
-      <c r="AJ134" t="inlineStr"/>
+      <c r="AI134" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ134" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK134" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -16663,8 +17727,16 @@
       <c r="AF135" t="inlineStr"/>
       <c r="AG135" t="inlineStr"/>
       <c r="AH135" t="inlineStr"/>
-      <c r="AI135" t="inlineStr"/>
-      <c r="AJ135" t="inlineStr"/>
+      <c r="AI135" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ135" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK135" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -16792,8 +17864,16 @@
       <c r="AF136" t="inlineStr"/>
       <c r="AG136" t="inlineStr"/>
       <c r="AH136" t="inlineStr"/>
-      <c r="AI136" t="inlineStr"/>
-      <c r="AJ136" t="inlineStr"/>
+      <c r="AI136" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ136" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK136" t="inlineStr">
         <is>
           <t>BELLARI</t>
@@ -16921,8 +18001,16 @@
       <c r="AF137" t="inlineStr"/>
       <c r="AG137" t="inlineStr"/>
       <c r="AH137" t="inlineStr"/>
-      <c r="AI137" t="inlineStr"/>
-      <c r="AJ137" t="inlineStr"/>
+      <c r="AI137" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ137" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK137" t="inlineStr">
         <is>
           <t>BELLARI</t>
@@ -17050,8 +18138,16 @@
       <c r="AF138" t="inlineStr"/>
       <c r="AG138" t="inlineStr"/>
       <c r="AH138" t="inlineStr"/>
-      <c r="AI138" t="inlineStr"/>
-      <c r="AJ138" t="inlineStr"/>
+      <c r="AI138" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ138" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK138" t="inlineStr">
         <is>
           <t>BELLARI</t>
@@ -17179,8 +18275,16 @@
       <c r="AF139" t="inlineStr"/>
       <c r="AG139" t="inlineStr"/>
       <c r="AH139" t="inlineStr"/>
-      <c r="AI139" t="inlineStr"/>
-      <c r="AJ139" t="inlineStr"/>
+      <c r="AI139" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ139" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK139" t="inlineStr">
         <is>
           <t>BELLARI</t>
@@ -17308,8 +18412,16 @@
       <c r="AF140" t="inlineStr"/>
       <c r="AG140" t="inlineStr"/>
       <c r="AH140" t="inlineStr"/>
-      <c r="AI140" t="inlineStr"/>
-      <c r="AJ140" t="inlineStr"/>
+      <c r="AI140" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ140" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK140" t="inlineStr">
         <is>
           <t>BELLARI</t>
@@ -17437,8 +18549,16 @@
       <c r="AF141" t="inlineStr"/>
       <c r="AG141" t="inlineStr"/>
       <c r="AH141" t="inlineStr"/>
-      <c r="AI141" t="inlineStr"/>
-      <c r="AJ141" t="inlineStr"/>
+      <c r="AI141" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ141" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK141" t="inlineStr"/>
       <c r="AL141" t="inlineStr"/>
       <c r="AM141" t="inlineStr"/>
@@ -17548,8 +18668,16 @@
       <c r="AF142" t="inlineStr"/>
       <c r="AG142" t="inlineStr"/>
       <c r="AH142" t="inlineStr"/>
-      <c r="AI142" t="inlineStr"/>
-      <c r="AJ142" t="inlineStr"/>
+      <c r="AI142" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ142" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK142" t="inlineStr"/>
       <c r="AL142" t="inlineStr"/>
       <c r="AM142" t="inlineStr"/>
@@ -17659,8 +18787,16 @@
       <c r="AF143" t="inlineStr"/>
       <c r="AG143" t="inlineStr"/>
       <c r="AH143" t="inlineStr"/>
-      <c r="AI143" t="inlineStr"/>
-      <c r="AJ143" t="inlineStr"/>
+      <c r="AI143" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ143" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK143" t="inlineStr"/>
       <c r="AL143" t="inlineStr"/>
       <c r="AM143" t="inlineStr"/>
@@ -17786,8 +18922,16 @@
       <c r="AF144" t="inlineStr"/>
       <c r="AG144" t="inlineStr"/>
       <c r="AH144" t="inlineStr"/>
-      <c r="AI144" t="inlineStr"/>
-      <c r="AJ144" t="inlineStr"/>
+      <c r="AI144" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ144" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK144" t="inlineStr"/>
       <c r="AL144" t="inlineStr"/>
       <c r="AM144" t="inlineStr"/>
@@ -17911,8 +19055,16 @@
       <c r="AF145" t="inlineStr"/>
       <c r="AG145" t="inlineStr"/>
       <c r="AH145" t="inlineStr"/>
-      <c r="AI145" t="inlineStr"/>
-      <c r="AJ145" t="inlineStr"/>
+      <c r="AI145" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ145" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK145" t="inlineStr"/>
       <c r="AL145" t="inlineStr"/>
       <c r="AM145" t="inlineStr"/>
@@ -18036,8 +19188,16 @@
       <c r="AF146" t="inlineStr"/>
       <c r="AG146" t="inlineStr"/>
       <c r="AH146" t="inlineStr"/>
-      <c r="AI146" t="inlineStr"/>
-      <c r="AJ146" t="inlineStr"/>
+      <c r="AI146" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ146" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK146" t="inlineStr">
         <is>
           <t>HO</t>
@@ -18165,8 +19325,16 @@
       <c r="AF147" t="inlineStr"/>
       <c r="AG147" t="inlineStr"/>
       <c r="AH147" t="inlineStr"/>
-      <c r="AI147" t="inlineStr"/>
-      <c r="AJ147" t="inlineStr"/>
+      <c r="AI147" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ147" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK147" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -18294,8 +19462,16 @@
       <c r="AF148" t="inlineStr"/>
       <c r="AG148" t="inlineStr"/>
       <c r="AH148" t="inlineStr"/>
-      <c r="AI148" t="inlineStr"/>
-      <c r="AJ148" t="inlineStr"/>
+      <c r="AI148" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ148" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK148" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -18423,8 +19599,16 @@
       <c r="AF149" t="inlineStr"/>
       <c r="AG149" t="inlineStr"/>
       <c r="AH149" t="inlineStr"/>
-      <c r="AI149" t="inlineStr"/>
-      <c r="AJ149" t="inlineStr"/>
+      <c r="AI149" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ149" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK149" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -18512,8 +19696,16 @@
       <c r="AF150" t="inlineStr"/>
       <c r="AG150" t="inlineStr"/>
       <c r="AH150" t="inlineStr"/>
-      <c r="AI150" t="inlineStr"/>
-      <c r="AJ150" t="inlineStr"/>
+      <c r="AI150" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ150" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK150" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -18641,8 +19833,16 @@
       <c r="AF151" t="inlineStr"/>
       <c r="AG151" t="inlineStr"/>
       <c r="AH151" t="inlineStr"/>
-      <c r="AI151" t="inlineStr"/>
-      <c r="AJ151" t="inlineStr"/>
+      <c r="AI151" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ151" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK151" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -18770,8 +19970,16 @@
       <c r="AF152" t="inlineStr"/>
       <c r="AG152" t="inlineStr"/>
       <c r="AH152" t="inlineStr"/>
-      <c r="AI152" t="inlineStr"/>
-      <c r="AJ152" t="inlineStr"/>
+      <c r="AI152" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ152" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK152" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -18899,8 +20107,16 @@
       <c r="AF153" t="inlineStr"/>
       <c r="AG153" t="inlineStr"/>
       <c r="AH153" t="inlineStr"/>
-      <c r="AI153" t="inlineStr"/>
-      <c r="AJ153" t="inlineStr"/>
+      <c r="AI153" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ153" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK153" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -19028,8 +20244,16 @@
       <c r="AF154" t="inlineStr"/>
       <c r="AG154" t="inlineStr"/>
       <c r="AH154" t="inlineStr"/>
-      <c r="AI154" t="inlineStr"/>
-      <c r="AJ154" t="inlineStr"/>
+      <c r="AI154" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ154" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK154" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -19157,8 +20381,16 @@
       <c r="AF155" t="inlineStr"/>
       <c r="AG155" t="inlineStr"/>
       <c r="AH155" t="inlineStr"/>
-      <c r="AI155" t="inlineStr"/>
-      <c r="AJ155" t="inlineStr"/>
+      <c r="AI155" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ155" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK155" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -19286,8 +20518,16 @@
       <c r="AF156" t="inlineStr"/>
       <c r="AG156" t="inlineStr"/>
       <c r="AH156" t="inlineStr"/>
-      <c r="AI156" t="inlineStr"/>
-      <c r="AJ156" t="inlineStr"/>
+      <c r="AI156" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ156" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK156" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -19415,8 +20655,16 @@
       <c r="AF157" t="inlineStr"/>
       <c r="AG157" t="inlineStr"/>
       <c r="AH157" t="inlineStr"/>
-      <c r="AI157" t="inlineStr"/>
-      <c r="AJ157" t="inlineStr"/>
+      <c r="AI157" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ157" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK157" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -19544,8 +20792,16 @@
       <c r="AF158" t="inlineStr"/>
       <c r="AG158" t="inlineStr"/>
       <c r="AH158" t="inlineStr"/>
-      <c r="AI158" t="inlineStr"/>
-      <c r="AJ158" t="inlineStr"/>
+      <c r="AI158" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ158" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK158" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -19669,8 +20925,16 @@
       <c r="AF159" t="inlineStr"/>
       <c r="AG159" t="inlineStr"/>
       <c r="AH159" t="inlineStr"/>
-      <c r="AI159" t="inlineStr"/>
-      <c r="AJ159" t="inlineStr"/>
+      <c r="AI159" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ159" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK159" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -19784,8 +21048,16 @@
       <c r="AF160" t="inlineStr"/>
       <c r="AG160" t="inlineStr"/>
       <c r="AH160" t="inlineStr"/>
-      <c r="AI160" t="inlineStr"/>
-      <c r="AJ160" t="inlineStr"/>
+      <c r="AI160" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ160" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK160" t="inlineStr"/>
       <c r="AL160" t="inlineStr"/>
       <c r="AM160" t="inlineStr"/>
@@ -19895,8 +21167,16 @@
       <c r="AF161" t="inlineStr"/>
       <c r="AG161" t="inlineStr"/>
       <c r="AH161" t="inlineStr"/>
-      <c r="AI161" t="inlineStr"/>
-      <c r="AJ161" t="inlineStr"/>
+      <c r="AI161" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ161" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK161" t="inlineStr"/>
       <c r="AL161" t="inlineStr"/>
       <c r="AM161" t="inlineStr"/>
@@ -20008,8 +21288,16 @@
       <c r="AF162" t="inlineStr"/>
       <c r="AG162" t="inlineStr"/>
       <c r="AH162" t="inlineStr"/>
-      <c r="AI162" t="inlineStr"/>
-      <c r="AJ162" t="inlineStr"/>
+      <c r="AI162" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ162" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK162" t="inlineStr"/>
       <c r="AL162" t="inlineStr"/>
       <c r="AM162" t="inlineStr"/>
@@ -20119,8 +21407,16 @@
       <c r="AF163" t="inlineStr"/>
       <c r="AG163" t="inlineStr"/>
       <c r="AH163" t="inlineStr"/>
-      <c r="AI163" t="inlineStr"/>
-      <c r="AJ163" t="inlineStr"/>
+      <c r="AI163" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ163" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK163" t="inlineStr"/>
       <c r="AL163" t="inlineStr"/>
       <c r="AM163" t="inlineStr"/>
@@ -20242,8 +21538,16 @@
       <c r="AF164" t="inlineStr"/>
       <c r="AG164" t="inlineStr"/>
       <c r="AH164" t="inlineStr"/>
-      <c r="AI164" t="inlineStr"/>
-      <c r="AJ164" t="inlineStr"/>
+      <c r="AI164" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ164" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK164" t="inlineStr"/>
       <c r="AL164" t="inlineStr"/>
       <c r="AM164" t="inlineStr"/>
@@ -20367,8 +21671,16 @@
       <c r="AF165" t="inlineStr"/>
       <c r="AG165" t="inlineStr"/>
       <c r="AH165" t="inlineStr"/>
-      <c r="AI165" t="inlineStr"/>
-      <c r="AJ165" t="inlineStr"/>
+      <c r="AI165" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ165" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK165" t="inlineStr">
         <is>
           <t>KOLKATA</t>
@@ -20496,8 +21808,16 @@
       <c r="AF166" t="inlineStr"/>
       <c r="AG166" t="inlineStr"/>
       <c r="AH166" t="inlineStr"/>
-      <c r="AI166" t="inlineStr"/>
-      <c r="AJ166" t="inlineStr"/>
+      <c r="AI166" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ166" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK166" t="inlineStr"/>
       <c r="AL166" t="inlineStr"/>
       <c r="AM166" t="inlineStr"/>
@@ -20621,8 +21941,16 @@
       <c r="AF167" t="inlineStr"/>
       <c r="AG167" t="inlineStr"/>
       <c r="AH167" t="inlineStr"/>
-      <c r="AI167" t="inlineStr"/>
-      <c r="AJ167" t="inlineStr"/>
+      <c r="AI167" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ167" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK167" t="inlineStr">
         <is>
           <t>BELLARI</t>
@@ -20750,8 +22078,16 @@
       <c r="AF168" t="inlineStr"/>
       <c r="AG168" t="inlineStr"/>
       <c r="AH168" t="inlineStr"/>
-      <c r="AI168" t="inlineStr"/>
-      <c r="AJ168" t="inlineStr"/>
+      <c r="AI168" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ168" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK168" t="inlineStr"/>
       <c r="AL168" t="inlineStr"/>
       <c r="AM168" t="inlineStr"/>
@@ -20875,8 +22211,16 @@
       <c r="AF169" t="inlineStr"/>
       <c r="AG169" t="inlineStr"/>
       <c r="AH169" t="inlineStr"/>
-      <c r="AI169" t="inlineStr"/>
-      <c r="AJ169" t="inlineStr"/>
+      <c r="AI169" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ169" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK169" t="inlineStr"/>
       <c r="AL169" t="inlineStr"/>
       <c r="AM169" t="inlineStr"/>
@@ -20986,8 +22330,16 @@
       <c r="AF170" t="inlineStr"/>
       <c r="AG170" t="inlineStr"/>
       <c r="AH170" t="inlineStr"/>
-      <c r="AI170" t="inlineStr"/>
-      <c r="AJ170" t="inlineStr"/>
+      <c r="AI170" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ170" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK170" t="inlineStr"/>
       <c r="AL170" t="inlineStr"/>
       <c r="AM170" t="inlineStr"/>
@@ -21097,8 +22449,16 @@
       <c r="AF171" t="inlineStr"/>
       <c r="AG171" t="inlineStr"/>
       <c r="AH171" t="inlineStr"/>
-      <c r="AI171" t="inlineStr"/>
-      <c r="AJ171" t="inlineStr"/>
+      <c r="AI171" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ171" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK171" t="inlineStr"/>
       <c r="AL171" t="inlineStr"/>
       <c r="AM171" t="inlineStr"/>
@@ -21208,8 +22568,16 @@
       <c r="AF172" t="inlineStr"/>
       <c r="AG172" t="inlineStr"/>
       <c r="AH172" t="inlineStr"/>
-      <c r="AI172" t="inlineStr"/>
-      <c r="AJ172" t="inlineStr"/>
+      <c r="AI172" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ172" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK172" t="inlineStr"/>
       <c r="AL172" t="inlineStr"/>
       <c r="AM172" t="inlineStr"/>
@@ -21335,8 +22703,16 @@
       <c r="AF173" t="inlineStr"/>
       <c r="AG173" t="inlineStr"/>
       <c r="AH173" t="inlineStr"/>
-      <c r="AI173" t="inlineStr"/>
-      <c r="AJ173" t="inlineStr"/>
+      <c r="AI173" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ173" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK173" t="inlineStr"/>
       <c r="AL173" t="inlineStr"/>
       <c r="AM173" t="inlineStr"/>
@@ -21450,8 +22826,16 @@
       <c r="AF174" t="inlineStr"/>
       <c r="AG174" t="inlineStr"/>
       <c r="AH174" t="inlineStr"/>
-      <c r="AI174" t="inlineStr"/>
-      <c r="AJ174" t="inlineStr"/>
+      <c r="AI174" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ174" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK174" t="inlineStr"/>
       <c r="AL174" t="inlineStr"/>
       <c r="AM174" t="inlineStr"/>
@@ -21565,8 +22949,16 @@
       <c r="AF175" t="inlineStr"/>
       <c r="AG175" t="inlineStr"/>
       <c r="AH175" t="inlineStr"/>
-      <c r="AI175" t="inlineStr"/>
-      <c r="AJ175" t="inlineStr"/>
+      <c r="AI175" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ175" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK175" t="inlineStr"/>
       <c r="AL175" t="inlineStr"/>
       <c r="AM175" t="inlineStr"/>
@@ -21680,8 +23072,16 @@
       <c r="AF176" t="inlineStr"/>
       <c r="AG176" t="inlineStr"/>
       <c r="AH176" t="inlineStr"/>
-      <c r="AI176" t="inlineStr"/>
-      <c r="AJ176" t="inlineStr"/>
+      <c r="AI176" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ176" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK176" t="inlineStr"/>
       <c r="AL176" t="inlineStr"/>
       <c r="AM176" t="inlineStr"/>
@@ -21795,8 +23195,16 @@
       <c r="AF177" t="inlineStr"/>
       <c r="AG177" t="inlineStr"/>
       <c r="AH177" t="inlineStr"/>
-      <c r="AI177" t="inlineStr"/>
-      <c r="AJ177" t="inlineStr"/>
+      <c r="AI177" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ177" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK177" t="inlineStr"/>
       <c r="AL177" t="inlineStr"/>
       <c r="AM177" t="inlineStr"/>
@@ -21910,8 +23318,16 @@
       <c r="AF178" t="inlineStr"/>
       <c r="AG178" t="inlineStr"/>
       <c r="AH178" t="inlineStr"/>
-      <c r="AI178" t="inlineStr"/>
-      <c r="AJ178" t="inlineStr"/>
+      <c r="AI178" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ178" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK178" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -22029,8 +23445,16 @@
       <c r="AF179" t="inlineStr"/>
       <c r="AG179" t="inlineStr"/>
       <c r="AH179" t="inlineStr"/>
-      <c r="AI179" t="inlineStr"/>
-      <c r="AJ179" t="inlineStr"/>
+      <c r="AI179" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
+      <c r="AJ179" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
       <c r="AK179" t="inlineStr"/>
       <c r="AL179" t="inlineStr"/>
       <c r="AM179" t="inlineStr"/>
@@ -22144,8 +23568,16 @@
       <c r="AF180" t="inlineStr"/>
       <c r="AG180" t="inlineStr"/>
       <c r="AH180" t="inlineStr"/>
-      <c r="AI180" t="inlineStr"/>
-      <c r="AJ180" t="inlineStr"/>
+      <c r="AI180" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ180" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK180" t="inlineStr"/>
       <c r="AL180" t="inlineStr"/>
       <c r="AM180" t="inlineStr"/>
@@ -22259,8 +23691,16 @@
       <c r="AF181" t="inlineStr"/>
       <c r="AG181" t="inlineStr"/>
       <c r="AH181" t="inlineStr"/>
-      <c r="AI181" t="inlineStr"/>
-      <c r="AJ181" t="inlineStr"/>
+      <c r="AI181" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ181" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK181" t="inlineStr"/>
       <c r="AL181" t="inlineStr"/>
       <c r="AM181" t="inlineStr"/>
@@ -22374,8 +23814,16 @@
       <c r="AF182" t="inlineStr"/>
       <c r="AG182" t="inlineStr"/>
       <c r="AH182" t="inlineStr"/>
-      <c r="AI182" t="inlineStr"/>
-      <c r="AJ182" t="inlineStr"/>
+      <c r="AI182" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ182" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK182" t="inlineStr"/>
       <c r="AL182" t="inlineStr"/>
       <c r="AM182" t="inlineStr"/>
@@ -22489,8 +23937,16 @@
       <c r="AF183" t="inlineStr"/>
       <c r="AG183" t="inlineStr"/>
       <c r="AH183" t="inlineStr"/>
-      <c r="AI183" t="inlineStr"/>
-      <c r="AJ183" t="inlineStr"/>
+      <c r="AI183" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ183" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK183" t="inlineStr"/>
       <c r="AL183" t="inlineStr"/>
       <c r="AM183" t="inlineStr"/>
@@ -22604,8 +24060,16 @@
       <c r="AF184" t="inlineStr"/>
       <c r="AG184" t="inlineStr"/>
       <c r="AH184" t="inlineStr"/>
-      <c r="AI184" t="inlineStr"/>
-      <c r="AJ184" t="inlineStr"/>
+      <c r="AI184" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ184" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK184" t="inlineStr"/>
       <c r="AL184" t="inlineStr"/>
       <c r="AM184" t="inlineStr"/>
@@ -22719,8 +24183,16 @@
       <c r="AF185" t="inlineStr"/>
       <c r="AG185" t="inlineStr"/>
       <c r="AH185" t="inlineStr"/>
-      <c r="AI185" t="inlineStr"/>
-      <c r="AJ185" t="inlineStr"/>
+      <c r="AI185" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ185" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK185" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -22850,8 +24322,16 @@
       <c r="AF186" t="inlineStr"/>
       <c r="AG186" t="inlineStr"/>
       <c r="AH186" t="inlineStr"/>
-      <c r="AI186" t="inlineStr"/>
-      <c r="AJ186" t="inlineStr"/>
+      <c r="AI186" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
+      <c r="AJ186" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
       <c r="AK186" t="inlineStr"/>
       <c r="AL186" t="inlineStr"/>
       <c r="AM186" t="inlineStr"/>
@@ -22965,8 +24445,16 @@
       <c r="AF187" t="inlineStr"/>
       <c r="AG187" t="inlineStr"/>
       <c r="AH187" t="inlineStr"/>
-      <c r="AI187" t="inlineStr"/>
-      <c r="AJ187" t="inlineStr"/>
+      <c r="AI187" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
+      <c r="AJ187" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
       <c r="AK187" t="inlineStr"/>
       <c r="AL187" t="inlineStr"/>
       <c r="AM187" t="inlineStr"/>
@@ -23080,8 +24568,16 @@
       <c r="AF188" t="inlineStr"/>
       <c r="AG188" t="inlineStr"/>
       <c r="AH188" t="inlineStr"/>
-      <c r="AI188" t="inlineStr"/>
-      <c r="AJ188" t="inlineStr"/>
+      <c r="AI188" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
+      <c r="AJ188" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
       <c r="AK188" t="inlineStr"/>
       <c r="AL188" t="inlineStr"/>
       <c r="AM188" t="inlineStr"/>
@@ -23205,8 +24701,16 @@
       <c r="AF189" t="inlineStr"/>
       <c r="AG189" t="inlineStr"/>
       <c r="AH189" t="inlineStr"/>
-      <c r="AI189" t="inlineStr"/>
-      <c r="AJ189" t="inlineStr"/>
+      <c r="AI189" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ189" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK189" t="inlineStr"/>
       <c r="AL189" t="inlineStr"/>
       <c r="AM189" t="inlineStr"/>
@@ -23330,8 +24834,16 @@
       <c r="AF190" t="inlineStr"/>
       <c r="AG190" t="inlineStr"/>
       <c r="AH190" t="inlineStr"/>
-      <c r="AI190" t="inlineStr"/>
-      <c r="AJ190" t="inlineStr"/>
+      <c r="AI190" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ190" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK190" t="inlineStr">
         <is>
           <t>HO</t>
@@ -23459,8 +24971,16 @@
       <c r="AF191" t="inlineStr"/>
       <c r="AG191" t="inlineStr"/>
       <c r="AH191" t="inlineStr"/>
-      <c r="AI191" t="inlineStr"/>
-      <c r="AJ191" t="inlineStr"/>
+      <c r="AI191" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ191" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK191" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -23588,8 +25108,16 @@
       <c r="AF192" t="inlineStr"/>
       <c r="AG192" t="inlineStr"/>
       <c r="AH192" t="inlineStr"/>
-      <c r="AI192" t="inlineStr"/>
-      <c r="AJ192" t="inlineStr"/>
+      <c r="AI192" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ192" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK192" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -23717,8 +25245,16 @@
       <c r="AF193" t="inlineStr"/>
       <c r="AG193" t="inlineStr"/>
       <c r="AH193" t="inlineStr"/>
-      <c r="AI193" t="inlineStr"/>
-      <c r="AJ193" t="inlineStr"/>
+      <c r="AI193" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ193" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK193" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -23806,8 +25342,16 @@
       <c r="AF194" t="inlineStr"/>
       <c r="AG194" t="inlineStr"/>
       <c r="AH194" t="inlineStr"/>
-      <c r="AI194" t="inlineStr"/>
-      <c r="AJ194" t="inlineStr"/>
+      <c r="AI194" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ194" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK194" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -23935,8 +25479,16 @@
       <c r="AF195" t="inlineStr"/>
       <c r="AG195" t="inlineStr"/>
       <c r="AH195" t="inlineStr"/>
-      <c r="AI195" t="inlineStr"/>
-      <c r="AJ195" t="inlineStr"/>
+      <c r="AI195" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ195" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK195" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -24064,8 +25616,16 @@
       <c r="AF196" t="inlineStr"/>
       <c r="AG196" t="inlineStr"/>
       <c r="AH196" t="inlineStr"/>
-      <c r="AI196" t="inlineStr"/>
-      <c r="AJ196" t="inlineStr"/>
+      <c r="AI196" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ196" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK196" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -24193,8 +25753,16 @@
       <c r="AF197" t="inlineStr"/>
       <c r="AG197" t="inlineStr"/>
       <c r="AH197" t="inlineStr"/>
-      <c r="AI197" t="inlineStr"/>
-      <c r="AJ197" t="inlineStr"/>
+      <c r="AI197" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ197" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK197" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -24322,8 +25890,16 @@
       <c r="AF198" t="inlineStr"/>
       <c r="AG198" t="inlineStr"/>
       <c r="AH198" t="inlineStr"/>
-      <c r="AI198" t="inlineStr"/>
-      <c r="AJ198" t="inlineStr"/>
+      <c r="AI198" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ198" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK198" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -24451,8 +26027,16 @@
       <c r="AF199" t="inlineStr"/>
       <c r="AG199" t="inlineStr"/>
       <c r="AH199" t="inlineStr"/>
-      <c r="AI199" t="inlineStr"/>
-      <c r="AJ199" t="inlineStr"/>
+      <c r="AI199" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ199" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK199" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -24580,8 +26164,16 @@
       <c r="AF200" t="inlineStr"/>
       <c r="AG200" t="inlineStr"/>
       <c r="AH200" t="inlineStr"/>
-      <c r="AI200" t="inlineStr"/>
-      <c r="AJ200" t="inlineStr"/>
+      <c r="AI200" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ200" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK200" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -24709,8 +26301,16 @@
       <c r="AF201" t="inlineStr"/>
       <c r="AG201" t="inlineStr"/>
       <c r="AH201" t="inlineStr"/>
-      <c r="AI201" t="inlineStr"/>
-      <c r="AJ201" t="inlineStr"/>
+      <c r="AI201" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ201" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK201" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -24838,8 +26438,16 @@
       <c r="AF202" t="inlineStr"/>
       <c r="AG202" t="inlineStr"/>
       <c r="AH202" t="inlineStr"/>
-      <c r="AI202" t="inlineStr"/>
-      <c r="AJ202" t="inlineStr"/>
+      <c r="AI202" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ202" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK202" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -24963,8 +26571,16 @@
       <c r="AF203" t="inlineStr"/>
       <c r="AG203" t="inlineStr"/>
       <c r="AH203" t="inlineStr"/>
-      <c r="AI203" t="inlineStr"/>
-      <c r="AJ203" t="inlineStr"/>
+      <c r="AI203" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ203" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK203" t="inlineStr">
         <is>
           <t>GOA</t>
@@ -25092,8 +26708,16 @@
       <c r="AF204" t="inlineStr"/>
       <c r="AG204" t="inlineStr"/>
       <c r="AH204" t="inlineStr"/>
-      <c r="AI204" t="inlineStr"/>
-      <c r="AJ204" t="inlineStr"/>
+      <c r="AI204" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ204" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK204" t="inlineStr"/>
       <c r="AL204" t="inlineStr"/>
       <c r="AM204" t="inlineStr"/>
@@ -25217,8 +26841,16 @@
       <c r="AF205" t="inlineStr"/>
       <c r="AG205" t="inlineStr"/>
       <c r="AH205" t="inlineStr"/>
-      <c r="AI205" t="inlineStr"/>
-      <c r="AJ205" t="inlineStr"/>
+      <c r="AI205" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ205" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK205" t="inlineStr">
         <is>
           <t>HO</t>
@@ -25334,8 +26966,16 @@
       <c r="AF206" t="inlineStr"/>
       <c r="AG206" t="inlineStr"/>
       <c r="AH206" t="inlineStr"/>
-      <c r="AI206" t="inlineStr"/>
-      <c r="AJ206" t="inlineStr"/>
+      <c r="AI206" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ206" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK206" t="inlineStr"/>
       <c r="AL206" t="inlineStr"/>
       <c r="AM206" t="inlineStr"/>
@@ -25459,8 +27099,16 @@
       <c r="AF207" t="inlineStr"/>
       <c r="AG207" t="inlineStr"/>
       <c r="AH207" t="inlineStr"/>
-      <c r="AI207" t="inlineStr"/>
-      <c r="AJ207" t="inlineStr"/>
+      <c r="AI207" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="AJ207" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
       <c r="AK207" t="inlineStr">
         <is>
           <t>BELLARI</t>
@@ -25588,8 +27236,16 @@
       <c r="AF208" t="inlineStr"/>
       <c r="AG208" t="inlineStr"/>
       <c r="AH208" t="inlineStr"/>
-      <c r="AI208" t="inlineStr"/>
-      <c r="AJ208" t="inlineStr"/>
+      <c r="AI208" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
+      <c r="AJ208" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
       <c r="AK208" t="inlineStr">
         <is>
           <t>BELLARI</t>
@@ -25717,8 +27373,16 @@
       <c r="AF209" t="inlineStr"/>
       <c r="AG209" t="inlineStr"/>
       <c r="AH209" t="inlineStr"/>
-      <c r="AI209" t="inlineStr"/>
-      <c r="AJ209" t="inlineStr"/>
+      <c r="AI209" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
+      <c r="AJ209" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
       <c r="AK209" t="inlineStr">
         <is>
           <t>HO</t>
@@ -25846,8 +27510,16 @@
       <c r="AF210" t="inlineStr"/>
       <c r="AG210" t="inlineStr"/>
       <c r="AH210" t="inlineStr"/>
-      <c r="AI210" t="inlineStr"/>
-      <c r="AJ210" t="inlineStr"/>
+      <c r="AI210" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
+      <c r="AJ210" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
       <c r="AK210" t="inlineStr">
         <is>
           <t>BELLARI</t>
@@ -25975,8 +27647,16 @@
       <c r="AF211" t="inlineStr"/>
       <c r="AG211" t="inlineStr"/>
       <c r="AH211" t="inlineStr"/>
-      <c r="AI211" t="inlineStr"/>
-      <c r="AJ211" t="inlineStr"/>
+      <c r="AI211" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
+      <c r="AJ211" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
       <c r="AK211" t="inlineStr">
         <is>
           <t>HO</t>
@@ -26104,8 +27784,16 @@
       <c r="AF212" t="inlineStr"/>
       <c r="AG212" t="inlineStr"/>
       <c r="AH212" t="inlineStr"/>
-      <c r="AI212" t="inlineStr"/>
-      <c r="AJ212" t="inlineStr"/>
+      <c r="AI212" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
+      <c r="AJ212" t="inlineStr">
+        <is>
+          <t>ACCEPTED</t>
+        </is>
+      </c>
       <c r="AK212" t="inlineStr"/>
       <c r="AL212" t="inlineStr"/>
       <c r="AM212" t="inlineStr"/>

</xml_diff>